<commit_message>
Initial commit for Magia Pilgrims
</commit_message>
<xml_diff>
--- a/files/CHR/ev_join.xlsx
+++ b/files/CHR/ev_join.xlsx
@@ -1,25 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\.antigravity\game\files\CHR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FCB708D-BBD1-4AEE-949B-C1ADA09B8A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D77CA6F9-72F1-4109-9808-74FD58D91918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1380" yWindow="585" windowWidth="26205" windowHeight="14895" xr2:uid="{C0E8C2FE-F33F-4C68-94BE-01501C7913C0}"/>
+    <workbookView xWindow="855" yWindow="225" windowWidth="26205" windowHeight="14850" xr2:uid="{C0E8C2FE-F33F-4C68-94BE-01501C7913C0}"/>
   </bookViews>
   <sheets>
-    <sheet name="009白蓮" sheetId="7" r:id="rId1"/>
-    <sheet name="3黄蘭" sheetId="2" r:id="rId2"/>
-    <sheet name="8紅華" sheetId="3" r:id="rId3"/>
-    <sheet name="11蒼樹" sheetId="4" r:id="rId4"/>
-    <sheet name="14李乃果" sheetId="5" r:id="rId5"/>
-    <sheet name="Sheet1" sheetId="6" r:id="rId6"/>
-    <sheet name="確認表" sheetId="1" r:id="rId7"/>
+    <sheet name="4ノア" sheetId="9" r:id="rId1"/>
+    <sheet name="009白蓮" sheetId="7" r:id="rId2"/>
+    <sheet name="0ななよ" sheetId="8" r:id="rId3"/>
+    <sheet name="3黄蘭" sheetId="2" r:id="rId4"/>
+    <sheet name="8紅華" sheetId="3" r:id="rId5"/>
+    <sheet name="11蒼樹" sheetId="4" r:id="rId6"/>
+    <sheet name="14李乃果" sheetId="5" r:id="rId7"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId8"/>
+    <sheet name="確認表" sheetId="1" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="343">
   <si>
     <t>愚者</t>
     <rPh sb="0" eb="2">
@@ -1458,6 +1460,266 @@
     <rPh sb="3" eb="5">
       <t>ドウコウ</t>
     </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>警戒は怠っていなかったはずだ。</t>
+  </si>
+  <si>
+    <t>だが、瓦礫の陰からその人影がふらりと現れた時、私は一瞬だけ引き金を引く指を止めてしまった。</t>
+  </si>
+  <si>
+    <t>こんな死と隣り合わせの地獄（タワー）のど真ん中で。</t>
+  </si>
+  <si>
+    <t>そいつは、まるで近所のコンビニにでも行くような足取りでこちらに歩み寄ってきたからだ。</t>
+  </si>
+  <si>
+    <t>「あ、すいませーん。ちょっと道、聞いてもいいですか？」</t>
+  </si>
+  <si>
+    <t>ふんわりとした、場違いなほど優しげな声。</t>
+  </si>
+  <si>
+    <t>振り返ると、頭に赤いハイビスカスの飾りをつけた少女が、にこにこと微笑んで立っていた。</t>
+  </si>
+  <si>
+    <t>「……えっ、だ、誰！何！？動かないで！」</t>
+  </si>
+  <si>
+    <t>「うわ、物騒やなぁ。私、ななよって言います。和歌山から来ました。怪しいもんやないですよ」</t>
+  </si>
+  <si>
+    <t>怪しいに決まっている。ここは化け物が徘徊する死地だ。</t>
+  </si>
+  <si>
+    <t>しかし、ななよと名乗った少女は、突きつけられた銃口を気にする素振りすら見せない。</t>
+  </si>
+  <si>
+    <t>「実は、友達を探してまして。この辺ではぐれちゃったみたいで」</t>
+  </si>
+  <si>
+    <t>「……ひ、人探し…？」</t>
+  </si>
+  <si>
+    <t>「はい！ ノアっていう子なんですけど、見ませんでした？」</t>
+  </si>
+  <si>
+    <t>張り詰めていた私の緊張が、少しだけ空回りする。</t>
+  </si>
+  <si>
+    <t>「……一応聞いておこうか、どんな子なの…？」</t>
+  </si>
+  <si>
+    <t>「ええとですね。小さくて、すっごく可愛い子なんです！」</t>
+  </si>
+  <si>
+    <t>「う、うん…」</t>
+  </si>
+  <si>
+    <t>「ちっちゃくて、こう、ぽわーっとしてて、とにかく可愛いんですよ！」</t>
+  </si>
+  <si>
+    <t>私は思わず天を仰ぎそうになった。</t>
+  </si>
+  <si>
+    <t>なんだその特徴は。主観の塊すぎて、欠片も手掛かりにならない。</t>
+  </si>
+  <si>
+    <t>「……そんな雑な特徴でわかるわけがないでしょう」</t>
+  </si>
+  <si>
+    <t>「えー、そうですかぁ……。絶対目立つと思うんやけどなぁ」</t>
+  </si>
+  <si>
+    <t>がっくりと肩を落とすななよに、私は警戒を解かないまま短く告げた。</t>
+  </si>
+  <si>
+    <t>「それらしい子には会ってないね、用が済んだなら、身を隠しなさい。ここは危ないよ」</t>
+  </si>
+  <si>
+    <t>背を向け、探索を再開しようと足を踏み出す。</t>
+  </si>
+  <si>
+    <t>だが、背後から無防備な足音が、トコトコとついてくるのが聞こえた。</t>
+  </si>
+  <si>
+    <t>「……なぜまだいる！」</t>
+  </si>
+  <si>
+    <t>「あ、もしよかったら、同行させてもらっていいですか？」</t>
+  </si>
+  <si>
+    <t>「ダメよ。ただでさえ危ないのにわけわかんない子まで連れて歩く余裕はないわ」</t>
+  </si>
+  <si>
+    <t>「えへへ、邪魔はしませんから。それに、一人でも多いほうが心強いでしょ？」</t>
+  </si>
+  <si>
+    <t>「ダメよ！勝手についてこないで！」</t>
+  </si>
+  <si>
+    <t>「あ、あそこの道、なんか危なそうな気配しますね。私が先に見に行ってきます！」</t>
+  </si>
+  <si>
+    <t>私の制止も聞かず、ななよは鼻歌でも歌い出しそうな軽やかさで前を歩き始めた。</t>
+  </si>
+  <si>
+    <t>緊張感という概念が完全に欠落している。</t>
+  </si>
+  <si>
+    <t>あまりのペースの違いに深いため息をつきながら、私は渋々、その背中を追う羽目になった。</t>
+  </si>
+  <si>
+    <t>狂気も、敵意も、絶望すらも感じられない。ただの、どこにでもいる女の子。</t>
+    <rPh sb="31" eb="32">
+      <t>オンナ</t>
+    </rPh>
+    <rPh sb="33" eb="34">
+      <t>コ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>私は銃口を下げないまま、声を絞り出す。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <t>[画像：evp007</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>.jpg</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ／ BGM：JOIN_US.mp3]</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>視線はずっと前から感じていた。 瓦礫の陰、崩れた柱の裏。一定の距離を保ちながら、何者かが私を執拗に観察している気配。 敵意はない。だが、ひどく怯えたような、迷うような視線だった。</t>
+  </si>
+  <si>
+    <t>私が銃を下ろし、あえて隙を見せて待っていると、やがて瓦礫の隙間からおずおずと小さな影が姿を現した。</t>
+  </si>
+  <si>
+    <t>「お、おい……そこの、お前」</t>
+  </si>
+  <si>
+    <t>声は微かに震えていた。 現れたのは、ひどく小柄で華奢な少女だった。 だが、その可憐な外見に反して、言葉遣いはやけに尊大で男性的だ。</t>
+  </si>
+  <si>
+    <t>虚勢を張って胸を反らせているが、華奢な肩は小刻みに震え、大きな瞳は不安げに揺らいでいる。 本来はプライドが高い性質なのだろう。だが、この絶望的な世界でたった一人、孤独と恐怖に耐え続けて限界を迎えているのは明白だった。</t>
+  </si>
+  <si>
+    <t>私はゆっくりと銃を地面に置き、両手を広げて一切の敵意がないことを示した。</t>
+  </si>
+  <si>
+    <t>私が極力声を落とし、ゆっくりと歩み寄ると、ノアはビクッと体をこわばらせた。 だが、逃げ出そうとはしなかった。 足元まで近づき、その小さな頭にそっと手を乗せる。</t>
+  </si>
+  <si>
+    <t>強張っていたノアの顔が、くしゃりと歪んだ。</t>
+  </si>
+  <si>
+    <t>「ぼ、ボクは……別に、怖くなんか……っ、うぅ……っ」 尊大な態度はとうに崩れ去っていた。 ノアは私の服の裾をぎゅっと強く握りしめ、小さな子供のように嗚咽を漏らし始めた。</t>
+  </si>
+  <si>
+    <t>私はその背中を、落ち着くまでただ優しく撫で続けた。 彼女がどれほどの時間を、この暗闇の中で一人震えて過ごしてきたのか、痛いほど分かったからだ。</t>
+  </si>
+  <si>
+    <t>ノアはまだ赤い目をこすりながら、こくりと小さく頷いた。 こうして、過酷なタワーの探索に、小さくて少し生意気な同行者が加わることになった。</t>
+  </si>
+  <si>
+    <t>「ボクの名はノア。……その、ずっと見ていたんだが、お前、なかなかやるじゃないか。ボ、ボクが特別に声をかけてやったんだ、光栄に思えよ」</t>
+    <rPh sb="4" eb="5">
+      <t>ナ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「えっ……」 「怖かったでしょう。偉かったね。もう大丈夫だよ」</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「ノア、私は紫苑」 やがて泣き止み、バツが悪そうに俯く彼女に、私はしゃがみ込んで目線を合わせ、穏やかに微笑みかけた。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「……お、お前が、どうしてもボクの力が必要だって言うなら……同行してやらないこともないぞ」</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">「私は今、人探しをしているんだ。……もし君さえよければ、私と一緒に来ない？」 </t>
+    <rPh sb="5" eb="7">
+      <t>ヒトサガ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「うん、必要だ。一人でも多ければ心強いよ。」</t>
+    <rPh sb="4" eb="6">
+      <t>ヒツヨウ</t>
+    </rPh>
+    <rPh sb="12" eb="13">
+      <t>オオ</t>
+    </rPh>
+    <rPh sb="16" eb="18">
+      <t>ココロヅヨ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">「……ノア、だね」 </t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「ひっ……な、なんだ。ボクに近づく気か！？」</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「大丈夫だ、取って食ったりしない。よく一人でここまで生き延びてきたね」</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <t>[画像：evp008</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>.jpg</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ／ BGM：JOIN_US.mp3]</t>
+    </r>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1949,6 +2211,127 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB1720EA-3884-4C74-9D88-634359EF668C}">
+  <dimension ref="A1:A36"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A4" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A6" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A8" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A14" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A16" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A18" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A19" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A20" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A21" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A23" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A25" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A27" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A29" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A31" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A33" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A34" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A35" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A36" t="s">
+        <v>332</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A525A19-3560-4B57-BB2F-740BEB71F838}">
   <dimension ref="A1:A91"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
@@ -2194,7 +2577,218 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1256C10E-4882-4971-97A7-D9028A3237C2}">
+  <dimension ref="A1:A53"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A4" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A5" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A6" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A7" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A13" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A15" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A16" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A17" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A19" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A20" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A22" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A23" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A24" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A26" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A27" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A28" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A29" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A30" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A32" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A33" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A35" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A36" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A38" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A39" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A41" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A42" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A44" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A45" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A46" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A47" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A48" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A49" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A51" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A52" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A53" t="s">
+        <v>318</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE20F5E2-AE2C-430F-B43B-A6A6CD4CD8A3}">
   <dimension ref="A1:A56"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
@@ -2395,7 +2989,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3469C594-26C7-4FE3-950B-14D575B86D76}">
   <dimension ref="A1:A52"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
@@ -2581,7 +3175,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBAF4A5B-E90A-48A1-872A-8298556D6D72}">
   <dimension ref="A1:A58"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
@@ -2782,7 +3376,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7155126A-5959-496C-8A1A-56FF633ADEB4}">
   <dimension ref="A1:A55"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
@@ -2958,7 +3552,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E7DFBF6-6D54-41E8-BB11-05C6A9B902E8}">
   <dimension ref="A1:T32"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
@@ -3162,7 +3756,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B16FA12E-9757-465B-9027-7E53794ED8E8}">
   <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>

</xml_diff>

<commit_message>
Deploy latest build to GitHub Pages
</commit_message>
<xml_diff>
--- a/files/CHR/ev_join.xlsx
+++ b/files/CHR/ev_join.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\.antigravity\game\files\CHR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D77CA6F9-72F1-4109-9808-74FD58D91918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34B68DA1-2F01-42EF-8599-4A19C7390026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="855" yWindow="225" windowWidth="26205" windowHeight="14850" xr2:uid="{C0E8C2FE-F33F-4C68-94BE-01501C7913C0}"/>
+    <workbookView xWindow="2025" yWindow="555" windowWidth="26205" windowHeight="14850" xr2:uid="{C0E8C2FE-F33F-4C68-94BE-01501C7913C0}"/>
   </bookViews>
   <sheets>
     <sheet name="4ノア" sheetId="9" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="355">
   <si>
     <t>愚者</t>
     <rPh sb="0" eb="2">
@@ -1612,90 +1612,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>視線はずっと前から感じていた。 瓦礫の陰、崩れた柱の裏。一定の距離を保ちながら、何者かが私を執拗に観察している気配。 敵意はない。だが、ひどく怯えたような、迷うような視線だった。</t>
-  </si>
-  <si>
-    <t>私が銃を下ろし、あえて隙を見せて待っていると、やがて瓦礫の隙間からおずおずと小さな影が姿を現した。</t>
-  </si>
-  <si>
-    <t>「お、おい……そこの、お前」</t>
-  </si>
-  <si>
-    <t>声は微かに震えていた。 現れたのは、ひどく小柄で華奢な少女だった。 だが、その可憐な外見に反して、言葉遣いはやけに尊大で男性的だ。</t>
-  </si>
-  <si>
-    <t>虚勢を張って胸を反らせているが、華奢な肩は小刻みに震え、大きな瞳は不安げに揺らいでいる。 本来はプライドが高い性質なのだろう。だが、この絶望的な世界でたった一人、孤独と恐怖に耐え続けて限界を迎えているのは明白だった。</t>
-  </si>
-  <si>
-    <t>私はゆっくりと銃を地面に置き、両手を広げて一切の敵意がないことを示した。</t>
-  </si>
-  <si>
-    <t>私が極力声を落とし、ゆっくりと歩み寄ると、ノアはビクッと体をこわばらせた。 だが、逃げ出そうとはしなかった。 足元まで近づき、その小さな頭にそっと手を乗せる。</t>
-  </si>
-  <si>
-    <t>強張っていたノアの顔が、くしゃりと歪んだ。</t>
-  </si>
-  <si>
-    <t>「ぼ、ボクは……別に、怖くなんか……っ、うぅ……っ」 尊大な態度はとうに崩れ去っていた。 ノアは私の服の裾をぎゅっと強く握りしめ、小さな子供のように嗚咽を漏らし始めた。</t>
-  </si>
-  <si>
-    <t>私はその背中を、落ち着くまでただ優しく撫で続けた。 彼女がどれほどの時間を、この暗闇の中で一人震えて過ごしてきたのか、痛いほど分かったからだ。</t>
-  </si>
-  <si>
-    <t>ノアはまだ赤い目をこすりながら、こくりと小さく頷いた。 こうして、過酷なタワーの探索に、小さくて少し生意気な同行者が加わることになった。</t>
-  </si>
-  <si>
-    <t>「ボクの名はノア。……その、ずっと見ていたんだが、お前、なかなかやるじゃないか。ボ、ボクが特別に声をかけてやったんだ、光栄に思えよ」</t>
-    <rPh sb="4" eb="5">
-      <t>ナ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>「えっ……」 「怖かったでしょう。偉かったね。もう大丈夫だよ」</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>「ノア、私は紫苑」 やがて泣き止み、バツが悪そうに俯く彼女に、私はしゃがみ込んで目線を合わせ、穏やかに微笑みかけた。</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>「……お、お前が、どうしてもボクの力が必要だって言うなら……同行してやらないこともないぞ」</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t xml:space="preserve">「私は今、人探しをしているんだ。……もし君さえよければ、私と一緒に来ない？」 </t>
-    <rPh sb="5" eb="7">
-      <t>ヒトサガ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>「うん、必要だ。一人でも多ければ心強いよ。」</t>
-    <rPh sb="4" eb="6">
-      <t>ヒツヨウ</t>
-    </rPh>
-    <rPh sb="12" eb="13">
-      <t>オオ</t>
-    </rPh>
-    <rPh sb="16" eb="18">
-      <t>ココロヅヨ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t xml:space="preserve">「……ノア、だね」 </t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>「ひっ……な、なんだ。ボクに近づく気か！？」</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>「大丈夫だ、取って食ったりしない。よく一人でここまで生き延びてきたね」</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <r>
       <t>[画像：evp008</t>
     </r>
@@ -1720,6 +1636,115 @@
       </rPr>
       <t xml:space="preserve"> ／ BGM：JOIN_US.mp3]</t>
     </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>返事はない。ただ、気配がさらに強張るのが分かった。</t>
+  </si>
+  <si>
+    <t>紫苑「大丈夫です。危害を加えたりしません」</t>
+  </si>
+  <si>
+    <t>紫苑は両手を広げた。</t>
+  </si>
+  <si>
+    <t>やがて瓦礫の陰から、大きな本を抱えた小さな人影が、警戒しながら姿を見せる。</t>
+  </si>
+  <si>
+    <t>——それを目にした瞬間、紫苑の声から硬さが抜けた。</t>
+  </si>
+  <si>
+    <t>紫苑「……名前、聞いてもいい?」</t>
+  </si>
+  <si>
+    <t>ノア「……ボクはノア」</t>
+  </si>
+  <si>
+    <t>紫苑「私は紫苑」</t>
+  </si>
+  <si>
+    <t>ノア「わけの分からないところに迷い込んで、連れとはぐれた。……何か知らないか」</t>
+  </si>
+  <si>
+    <t>紫苑「ごめん、私にも分からない」</t>
+  </si>
+  <si>
+    <t>ノア「……そうか」</t>
+  </si>
+  <si>
+    <t>その時、遠くで瓦礫が崩れる音がした。ノアの肩が大きく跳ねる。</t>
+  </si>
+  <si>
+    <t>ノア「……っ、今のは」</t>
+  </si>
+  <si>
+    <t>紫苑「たぶん、何かが崩れただけだよ」</t>
+  </si>
+  <si>
+    <t>ノア「どこかでまた化け物が…」</t>
+  </si>
+  <si>
+    <t>そう言う手は、本を強く握りしめていた。</t>
+  </si>
+  <si>
+    <t>紫苑「……怖いなら、怖いって言っていいんだよ」</t>
+  </si>
+  <si>
+    <t>ノア「……怖い、というのは、正確な表現じゃ……」</t>
+  </si>
+  <si>
+    <t>言葉が、そこで途切れた。強張っていた顔が、じわりと崩れていく。</t>
+  </si>
+  <si>
+    <t>ノア「……ずっと、考えて……それでも、追いつかなくて……」</t>
+  </si>
+  <si>
+    <t>立ち上がろうとした足が、瓦礫に取られてよろめく。</t>
+  </si>
+  <si>
+    <t>紫苑は咄嗟に、倒れかけたその体を抱きとめた。</t>
+  </si>
+  <si>
+    <t>腕の中は、驚くほど軽く、冷え切って、小さく震えていた。</t>
+  </si>
+  <si>
+    <t>紫苑はその体を、少し強く抱き寄せる。</t>
+  </si>
+  <si>
+    <t>紫苑「……怖かったんだね」</t>
+  </si>
+  <si>
+    <t>ノア「……っ……」</t>
+  </si>
+  <si>
+    <t>堪えていたものが、そこで決壊した。ノアは紫苑にしがみつき、声を上げて泣き始める。</t>
+  </si>
+  <si>
+    <t>紫苑は何も言わず、ただその背中を撫で続けた。</t>
+  </si>
+  <si>
+    <t>やがて、嗚咽が少しずつ収まっていく。</t>
+  </si>
+  <si>
+    <t>紫苑「……一緒に、友達を探そう」</t>
+  </si>
+  <si>
+    <t>ノア「……うん」</t>
+  </si>
+  <si>
+    <t>木々に覆われた廃墟の中、紫苑は微かな気配を感じ取った。呼吸の音。人間のものだ。</t>
+    <rPh sb="0" eb="2">
+      <t>キギ</t>
+    </rPh>
+    <rPh sb="3" eb="4">
+      <t>オオ</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>ハイキョ</t>
+    </rPh>
+    <rPh sb="10" eb="11">
+      <t>ナカ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -2212,7 +2237,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB1720EA-3884-4C74-9D88-634359EF668C}">
-  <dimension ref="A1:A36"/>
+  <dimension ref="A1:A68"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.4">
@@ -2222,32 +2247,32 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>342</v>
+        <v>322</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>322</v>
+        <v>354</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>323</v>
+        <v>239</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.4">
@@ -2262,52 +2287,42 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A19" t="s">
-        <v>340</v>
+        <v>328</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A21" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A23" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A22" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A24" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A26" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A28" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A30" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A25" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A27" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A29" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A31" t="s">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A32" t="s">
         <v>335</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A33" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.4">
@@ -2315,14 +2330,89 @@
         <v>336</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A35" t="s">
-        <v>338</v>
-      </c>
-    </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
-        <v>332</v>
+        <v>337</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A38" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A40" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A42" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A44" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A46" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A48" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A50" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A52" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A54" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A56" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A58" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A60" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A62" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A64" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A66" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A68" t="s">
+        <v>353</v>
       </c>
     </row>
   </sheetData>

</xml_diff>